<commit_message>
Minor commits after updating v2_lang_3groups_SUMMARY.qmd to add combined OR chart
</commit_message>
<xml_diff>
--- a/Data/race v.3.xlsx
+++ b/Data/race v.3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hata/Desktop/EDLD652_Diss/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maiko/Desktop/EDLD652_Diss/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A226EFC5-D23C-2245-9492-6B414BEAE610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF30F22-FF1C-E449-B491-D5D32D97A29B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="500" windowWidth="25400" windowHeight="15900" xr2:uid="{1EA0D511-E3B1-4D4B-AFF6-A41D55739002}"/>
+    <workbookView xWindow="13280" yWindow="820" windowWidth="25400" windowHeight="15900" xr2:uid="{1EA0D511-E3B1-4D4B-AFF6-A41D55739002}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -618,7 +618,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ACE525B-B2AD-9C4D-80D9-58F59817B9C0}">
-  <dimension ref="A1:N141"/>
+  <dimension ref="A1:N142"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:14" ht="98" x14ac:dyDescent="0.2">
@@ -6434,6 +6434,16 @@
       <c r="D141" s="14">
         <f>SUM(D72:D140)</f>
         <v>4949882</v>
+      </c>
+    </row>
+    <row r="142" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="G142" s="14">
+        <f>SUM(G132:G141)</f>
+        <v>3864</v>
+      </c>
+      <c r="L142" s="14">
+        <f>SUM(L132:L141)</f>
+        <v>55410</v>
       </c>
     </row>
   </sheetData>

</xml_diff>